<commit_message>
Update misclassification_distribution_with_family_flag.xlsx for improved data accuracy
</commit_message>
<xml_diff>
--- a/CSVs/misclassification_distribution_with_family_flag.xlsx
+++ b/CSVs/misclassification_distribution_with_family_flag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meghp\Desktop\Ahmedabad University\Term 1\CSE618 Artificial Intelligence Laboratory\Bird Species Detection\CSVs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E15217-3E78-4868-B83D-09F370B78880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A3A3F02-0525-47A0-A836-951902722685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BE3F7B11-DE27-46EE-97E8-441B81A35EB4}"/>
   </bookViews>
@@ -1336,7 +1336,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1354,16 +1354,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1751,19 +1741,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>118</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C4" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F4" s="4">
         <v>1</v>
@@ -1791,19 +1781,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C6" s="4">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F6" s="4">
         <v>1</v>
@@ -1931,19 +1921,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>34</v>
+        <v>156</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>35</v>
+        <v>157</v>
       </c>
       <c r="C13" s="4">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>36</v>
+        <v>158</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F13" s="4">
         <v>1</v>
@@ -1971,19 +1961,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>40</v>
+        <v>152</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>41</v>
+        <v>155</v>
       </c>
       <c r="C15" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>42</v>
+        <v>154</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>43</v>
+        <v>119</v>
       </c>
       <c r="F15" s="4">
         <v>1</v>
@@ -2091,19 +2081,19 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>50</v>
+        <v>152</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C21" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>51</v>
+        <v>154</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="F21" s="4">
         <v>1</v>
@@ -2111,19 +2101,19 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>20</v>
+        <v>153</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C22" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>22</v>
+        <v>154</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F22" s="4">
         <v>1</v>
@@ -2531,19 +2521,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C43" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
       <c r="F43" s="4">
         <v>1</v>
@@ -2671,19 +2661,19 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="C50" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>62</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="F50" s="4">
         <v>1</v>
@@ -2871,19 +2861,19 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C60" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>91</v>
+        <v>22</v>
       </c>
       <c r="F60" s="4">
         <v>1</v>
@@ -3031,19 +3021,19 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="C68" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="F68" s="4">
         <v>1</v>
@@ -3091,19 +3081,19 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>104</v>
+        <v>192</v>
       </c>
       <c r="C71" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>106</v>
+        <v>190</v>
       </c>
       <c r="F71" s="4">
         <v>1</v>
@@ -3111,19 +3101,19 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B72" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>107</v>
       </c>
       <c r="C72" s="4">
         <v>3</v>
       </c>
       <c r="D72" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E72" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="F72" s="4">
         <v>1</v>
@@ -3131,19 +3121,19 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>38</v>
+        <v>107</v>
       </c>
       <c r="C73" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="F73" s="4">
         <v>1</v>
@@ -3151,19 +3141,19 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>34</v>
+        <v>247</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="C74" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>36</v>
+        <v>248</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="F74" s="4">
         <v>1</v>
@@ -3251,19 +3241,19 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>33</v>
+        <v>214</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>19</v>
+        <v>113</v>
       </c>
       <c r="C79" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>21</v>
+        <v>115</v>
       </c>
       <c r="F79" s="4">
         <v>1</v>
@@ -3291,19 +3281,19 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>113</v>
+        <v>249</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>114</v>
+        <v>73</v>
       </c>
       <c r="C81" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>116</v>
+        <v>14</v>
       </c>
       <c r="F81" s="4">
         <v>1</v>
@@ -3311,19 +3301,19 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="C82" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="F82" s="4">
         <v>1</v>
@@ -3471,19 +3461,19 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>127</v>
+        <v>205</v>
       </c>
       <c r="C90" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>14</v>
+        <v>206</v>
       </c>
       <c r="F90" s="4">
         <v>1</v>
@@ -3591,19 +3581,19 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>128</v>
+        <v>25</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="C96" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="F96" s="4">
         <v>1</v>
@@ -3711,19 +3701,19 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>131</v>
+        <v>25</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="C102" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="F102" s="4">
         <v>1</v>
@@ -3751,19 +3741,19 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>118</v>
+        <v>55</v>
       </c>
       <c r="C104" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>133</v>
+        <v>27</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>119</v>
+        <v>57</v>
       </c>
       <c r="F104" s="4">
         <v>1</v>
@@ -3771,19 +3761,19 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
-        <v>107</v>
+        <v>26</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>61</v>
+        <v>200</v>
       </c>
       <c r="C105" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>62</v>
+        <v>201</v>
       </c>
       <c r="F105" s="4">
         <v>1</v>
@@ -3951,19 +3941,19 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>136</v>
+        <v>61</v>
       </c>
       <c r="C114" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="F114" s="4">
         <v>1</v>
@@ -3971,19 +3961,19 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
-        <v>19</v>
+        <v>193</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="C115" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="F115" s="4">
         <v>1</v>
@@ -3994,16 +3984,16 @@
         <v>80</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
       <c r="C116" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D116" s="4" t="s">
         <v>81</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="F116" s="4">
         <v>1</v>
@@ -4051,19 +4041,19 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>142</v>
+        <v>61</v>
       </c>
       <c r="C119" s="4">
         <v>2</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>143</v>
+        <v>62</v>
       </c>
       <c r="F119" s="4">
         <v>1</v>
@@ -4091,19 +4081,19 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C121" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F121" s="4">
         <v>1</v>
@@ -4111,19 +4101,19 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>124</v>
+        <v>207</v>
       </c>
       <c r="C122" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>139</v>
+        <v>81</v>
       </c>
       <c r="E122" s="4" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="F122" s="4">
         <v>1</v>
@@ -4151,19 +4141,19 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="C124" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>148</v>
+        <v>81</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="F124" s="4">
         <v>1</v>
@@ -4171,19 +4161,19 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>132</v>
+        <v>78</v>
       </c>
       <c r="C125" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>133</v>
+        <v>79</v>
       </c>
       <c r="F125" s="4">
         <v>1</v>
@@ -4291,19 +4281,19 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>132</v>
+        <v>19</v>
       </c>
       <c r="C131" s="4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>133</v>
+        <v>21</v>
       </c>
       <c r="F131" s="4">
         <v>1</v>
@@ -4311,19 +4301,19 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="4" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="C132" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="F132" s="4">
         <v>1</v>
@@ -4371,19 +4361,19 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="C135" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="F135" s="4">
         <v>1</v>
@@ -4451,19 +4441,19 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
-        <v>118</v>
+        <v>33</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C139" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>119</v>
+        <v>22</v>
       </c>
       <c r="E139" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F139" s="4">
         <v>1</v>
@@ -4471,19 +4461,19 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="4" t="s">
-        <v>118</v>
+        <v>33</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>58</v>
+        <v>107</v>
       </c>
       <c r="C140" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>119</v>
+        <v>22</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="F140" s="4">
         <v>1</v>
@@ -4511,19 +4501,19 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="4" t="s">
-        <v>156</v>
+        <v>33</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>157</v>
+        <v>193</v>
       </c>
       <c r="C142" s="4">
         <v>1</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>158</v>
+        <v>22</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="F142" s="4">
         <v>1</v>
@@ -4571,19 +4561,19 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="4" t="s">
-        <v>160</v>
+        <v>33</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>161</v>
+        <v>61</v>
       </c>
       <c r="C145" s="4">
         <v>1</v>
       </c>
       <c r="D145" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>162</v>
+        <v>62</v>
       </c>
       <c r="F145" s="4">
         <v>1</v>
@@ -4591,19 +4581,19 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="4" t="s">
-        <v>160</v>
+        <v>66</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>24</v>
+        <v>180</v>
       </c>
       <c r="C146" s="4">
         <v>1</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F146" s="4">
         <v>1</v>
@@ -4691,19 +4681,19 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="4" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C151" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>108</v>
+        <v>68</v>
       </c>
       <c r="E151" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F151" s="4">
         <v>1</v>
@@ -4711,19 +4701,19 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>167</v>
+        <v>227</v>
       </c>
       <c r="C152" s="4">
         <v>1</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>108</v>
+        <v>68</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>168</v>
+        <v>62</v>
       </c>
       <c r="F152" s="4">
         <v>1</v>
@@ -4791,19 +4781,19 @@
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B156" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B156" s="4" t="s">
-        <v>171</v>
-      </c>
       <c r="C156" s="4">
         <v>1</v>
       </c>
       <c r="D156" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E156" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="E156" s="4" t="s">
-        <v>172</v>
       </c>
       <c r="F156" s="4">
         <v>1</v>
@@ -4831,19 +4821,19 @@
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
-        <v>78</v>
+        <v>228</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="C158" s="4">
         <v>1</v>
       </c>
       <c r="D158" s="4" t="s">
-        <v>79</v>
+        <v>172</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>71</v>
+        <v>139</v>
       </c>
       <c r="F158" s="4">
         <v>1</v>
@@ -4911,19 +4901,19 @@
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>132</v>
+        <v>229</v>
       </c>
       <c r="C162" s="4">
         <v>1</v>
       </c>
       <c r="D162" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E162" s="4" t="s">
-        <v>133</v>
+        <v>204</v>
       </c>
       <c r="F162" s="4">
         <v>1</v>
@@ -4931,19 +4921,19 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C163" s="4">
         <v>1</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>176</v>
+        <v>37</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F163" s="4">
         <v>1</v>
@@ -4951,10 +4941,10 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
-        <v>39</v>
+        <v>238</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>13</v>
+        <v>220</v>
       </c>
       <c r="C164" s="4">
         <v>1</v>
@@ -4963,7 +4953,7 @@
         <v>37</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="F164" s="4">
         <v>1</v>
@@ -4991,19 +4981,19 @@
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
-        <v>177</v>
+        <v>38</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="C166" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D166" s="4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E166" s="4" t="s">
-        <v>8</v>
+        <v>101</v>
       </c>
       <c r="F166" s="4">
         <v>1</v>
@@ -5031,19 +5021,19 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="C168" s="4">
         <v>1</v>
       </c>
       <c r="D168" s="4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="F168" s="4">
         <v>1</v>
@@ -5051,19 +5041,19 @@
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="4" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>178</v>
+        <v>34</v>
       </c>
       <c r="C169" s="4">
         <v>1</v>
       </c>
       <c r="D169" s="4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E169" s="4" t="s">
-        <v>179</v>
+        <v>36</v>
       </c>
       <c r="F169" s="4">
         <v>1</v>
@@ -5071,19 +5061,19 @@
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="4" t="s">
-        <v>180</v>
+        <v>38</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>151</v>
+        <v>13</v>
       </c>
       <c r="C170" s="4">
         <v>1</v>
       </c>
       <c r="D170" s="4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E170" s="4" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="F170" s="4">
         <v>1</v>
@@ -5091,19 +5081,19 @@
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="4" t="s">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C171" s="4">
         <v>1</v>
       </c>
       <c r="D171" s="4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E171" s="4" t="s">
-        <v>182</v>
+        <v>14</v>
       </c>
       <c r="F171" s="4">
         <v>1</v>
@@ -5111,19 +5101,19 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" s="4" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C172" s="4">
         <v>1</v>
       </c>
       <c r="D172" s="4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E172" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F172" s="4">
         <v>1</v>
@@ -5131,19 +5121,19 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="C173" s="4">
         <v>1</v>
       </c>
       <c r="D173" s="4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E173" s="4" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="F173" s="4">
         <v>1</v>
@@ -5171,19 +5161,19 @@
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" s="4" t="s">
-        <v>184</v>
+        <v>35</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C175" s="4">
         <v>1</v>
       </c>
       <c r="D175" s="4" t="s">
-        <v>185</v>
+        <v>37</v>
       </c>
       <c r="E175" s="4" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="F175" s="4">
         <v>1</v>
@@ -5191,19 +5181,19 @@
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
-        <v>144</v>
+        <v>35</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>186</v>
+        <v>67</v>
       </c>
       <c r="C176" s="4">
         <v>1</v>
       </c>
       <c r="D176" s="4" t="s">
-        <v>146</v>
+        <v>37</v>
       </c>
       <c r="E176" s="4" t="s">
-        <v>187</v>
+        <v>68</v>
       </c>
       <c r="F176" s="4">
         <v>1</v>
@@ -5211,19 +5201,19 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" s="4" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="C177" s="4">
         <v>1</v>
       </c>
       <c r="D177" s="4" t="s">
-        <v>148</v>
+        <v>37</v>
       </c>
       <c r="E177" s="4" t="s">
-        <v>30</v>
+        <v>91</v>
       </c>
       <c r="F177" s="4">
         <v>1</v>
@@ -5231,19 +5221,19 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" s="4" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="C178" s="4">
         <v>1</v>
       </c>
       <c r="D178" s="4" t="s">
-        <v>148</v>
+        <v>37</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>190</v>
+        <v>14</v>
       </c>
       <c r="F178" s="4">
         <v>1</v>
@@ -5251,19 +5241,19 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" s="4" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>50</v>
+        <v>124</v>
       </c>
       <c r="C179" s="4">
         <v>1</v>
       </c>
       <c r="D179" s="4" t="s">
-        <v>148</v>
+        <v>37</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="F179" s="4">
         <v>1</v>
@@ -5271,19 +5261,19 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" s="4" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="C180" s="4">
         <v>1</v>
       </c>
       <c r="D180" s="4" t="s">
-        <v>148</v>
+        <v>37</v>
       </c>
       <c r="E180" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F180" s="4">
         <v>1</v>
@@ -5291,19 +5281,19 @@
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" s="4" t="s">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>102</v>
+        <v>222</v>
       </c>
       <c r="C181" s="4">
         <v>1</v>
       </c>
       <c r="D181" s="4" t="s">
-        <v>148</v>
+        <v>37</v>
       </c>
       <c r="E181" s="4" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="F181" s="4">
         <v>1</v>
@@ -5311,19 +5301,19 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" s="4" t="s">
-        <v>147</v>
+        <v>223</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>191</v>
+        <v>16</v>
       </c>
       <c r="C182" s="4">
         <v>1</v>
       </c>
       <c r="D182" s="4" t="s">
-        <v>148</v>
+        <v>224</v>
       </c>
       <c r="E182" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F182" s="4">
         <v>1</v>
@@ -5331,19 +5321,19 @@
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="C183" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D183" s="4" t="s">
-        <v>65</v>
+        <v>133</v>
       </c>
       <c r="E183" s="4" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="F183" s="4">
         <v>1</v>
@@ -5351,19 +5341,19 @@
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
-        <v>16</v>
+        <v>132</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>29</v>
+        <v>155</v>
       </c>
       <c r="C184" s="4">
         <v>1</v>
       </c>
       <c r="D184" s="4" t="s">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="E184" s="4" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="F184" s="4">
         <v>1</v>
@@ -5371,19 +5361,19 @@
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" s="4" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>155</v>
+        <v>16</v>
       </c>
       <c r="C185" s="4">
         <v>1</v>
       </c>
       <c r="D185" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E185" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="E185" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="F185" s="4">
         <v>1</v>
@@ -5391,19 +5381,19 @@
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
-        <v>17</v>
+        <v>107</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="C186" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D186" s="4" t="s">
-        <v>18</v>
+        <v>108</v>
       </c>
       <c r="E186" s="4" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="F186" s="4">
         <v>1</v>
@@ -5491,19 +5481,19 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" s="4" t="s">
-        <v>28</v>
+        <v>107</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>175</v>
+        <v>33</v>
       </c>
       <c r="C191" s="4">
         <v>1</v>
       </c>
       <c r="D191" s="4" t="s">
-        <v>30</v>
+        <v>108</v>
       </c>
       <c r="E191" s="4" t="s">
-        <v>176</v>
+        <v>22</v>
       </c>
       <c r="F191" s="4">
         <v>1</v>
@@ -5511,19 +5501,19 @@
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" s="4" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="C192" s="4">
         <v>1</v>
       </c>
       <c r="D192" s="4" t="s">
-        <v>30</v>
+        <v>108</v>
       </c>
       <c r="E192" s="4" t="s">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="F192" s="4">
         <v>1</v>
@@ -5531,19 +5521,19 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
-        <v>33</v>
+        <v>107</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>193</v>
+        <v>60</v>
       </c>
       <c r="C193" s="4">
         <v>1</v>
       </c>
       <c r="D193" s="4" t="s">
-        <v>22</v>
+        <v>108</v>
       </c>
       <c r="E193" s="4" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="F193" s="4">
         <v>1</v>
@@ -5551,19 +5541,19 @@
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" s="4" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C194" s="4">
         <v>1</v>
       </c>
       <c r="D194" s="4" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="E194" s="4" t="s">
-        <v>14</v>
+        <v>182</v>
       </c>
       <c r="F194" s="4">
         <v>1</v>
@@ -5611,19 +5601,19 @@
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" s="4" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="C197" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D197" s="4" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="E197" s="4" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F197" s="4">
         <v>1</v>
@@ -5631,19 +5621,19 @@
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>100</v>
+        <v>171</v>
       </c>
       <c r="C198" s="4">
         <v>1</v>
       </c>
       <c r="D198" s="4" t="s">
-        <v>195</v>
+        <v>115</v>
       </c>
       <c r="E198" s="4" t="s">
-        <v>101</v>
+        <v>172</v>
       </c>
       <c r="F198" s="4">
         <v>1</v>
@@ -5651,19 +5641,19 @@
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" s="4" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="C199" s="4">
         <v>1</v>
       </c>
       <c r="D199" s="4" t="s">
-        <v>195</v>
+        <v>115</v>
       </c>
       <c r="E199" s="4" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F199" s="4">
         <v>1</v>
@@ -5671,19 +5661,19 @@
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" s="4" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>180</v>
+        <v>153</v>
       </c>
       <c r="C200" s="4">
         <v>1</v>
       </c>
       <c r="D200" s="4" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="E200" s="4" t="s">
-        <v>14</v>
+        <v>154</v>
       </c>
       <c r="F200" s="4">
         <v>1</v>
@@ -5691,19 +5681,19 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B201" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B201" s="4" t="s">
-        <v>7</v>
-      </c>
       <c r="C201" s="4">
         <v>1</v>
       </c>
       <c r="D201" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E201" s="4" t="s">
         <v>176</v>
-      </c>
-      <c r="E201" s="4" t="s">
-        <v>8</v>
       </c>
       <c r="F201" s="4">
         <v>1</v>
@@ -5711,19 +5701,19 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" s="4" t="s">
-        <v>196</v>
+        <v>28</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="C202" s="4">
         <v>1</v>
       </c>
       <c r="D202" s="4" t="s">
-        <v>197</v>
+        <v>30</v>
       </c>
       <c r="E202" s="4" t="s">
-        <v>71</v>
+        <v>133</v>
       </c>
       <c r="F202" s="4">
         <v>1</v>
@@ -5731,19 +5721,19 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
-        <v>198</v>
+        <v>49</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="C203" s="4">
         <v>1</v>
       </c>
       <c r="D203" s="4" t="s">
-        <v>199</v>
+        <v>30</v>
       </c>
       <c r="E203" s="4" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="F203" s="4">
         <v>1</v>
@@ -5751,19 +5741,19 @@
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" s="4" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>17</v>
+        <v>128</v>
       </c>
       <c r="C204" s="4">
         <v>1</v>
       </c>
       <c r="D204" s="4" t="s">
-        <v>199</v>
+        <v>30</v>
       </c>
       <c r="E204" s="4" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F204" s="4">
         <v>1</v>
@@ -5771,19 +5761,19 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" s="4" t="s">
-        <v>200</v>
+        <v>54</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="C205" s="4">
         <v>1</v>
       </c>
       <c r="D205" s="4" t="s">
-        <v>201</v>
+        <v>30</v>
       </c>
       <c r="E205" s="4" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="F205" s="4">
         <v>1</v>
@@ -5791,19 +5781,19 @@
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" s="4" t="s">
-        <v>200</v>
+        <v>54</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="C206" s="4">
         <v>1</v>
       </c>
       <c r="D206" s="4" t="s">
-        <v>201</v>
+        <v>30</v>
       </c>
       <c r="E206" s="4" t="s">
-        <v>146</v>
+        <v>179</v>
       </c>
       <c r="F206" s="4">
         <v>1</v>
@@ -5851,19 +5841,19 @@
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" s="4" t="s">
-        <v>141</v>
+        <v>48</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="C209" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D209" s="4" t="s">
-        <v>139</v>
+        <v>30</v>
       </c>
       <c r="E209" s="4" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="F209" s="4">
         <v>1</v>
@@ -5891,19 +5881,19 @@
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" s="4" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="C211" s="4">
         <v>1</v>
       </c>
       <c r="D211" s="4" t="s">
-        <v>139</v>
+        <v>65</v>
       </c>
       <c r="E211" s="4" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="F211" s="4">
         <v>1</v>
@@ -5911,19 +5901,19 @@
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" s="4" t="s">
-        <v>137</v>
+        <v>64</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>12</v>
+        <v>142</v>
       </c>
       <c r="C212" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D212" s="4" t="s">
-        <v>139</v>
+        <v>65</v>
       </c>
       <c r="E212" s="4" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="F212" s="4">
         <v>1</v>
@@ -5951,19 +5941,19 @@
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" s="4" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>41</v>
+        <v>142</v>
       </c>
       <c r="C214" s="4">
         <v>1</v>
       </c>
       <c r="D214" s="4" t="s">
-        <v>139</v>
+        <v>65</v>
       </c>
       <c r="E214" s="4" t="s">
-        <v>43</v>
+        <v>143</v>
       </c>
       <c r="F214" s="4">
         <v>1</v>
@@ -6011,19 +6001,19 @@
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" s="4" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C217" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D217" s="4" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="E217" s="4" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F217" s="4">
         <v>1</v>
@@ -6051,19 +6041,19 @@
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219" s="4" t="s">
-        <v>202</v>
+        <v>16</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>203</v>
+        <v>29</v>
       </c>
       <c r="C219" s="4">
         <v>1</v>
       </c>
       <c r="D219" s="4" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="E219" s="4" t="s">
-        <v>204</v>
+        <v>30</v>
       </c>
       <c r="F219" s="4">
         <v>1</v>
@@ -6071,19 +6061,19 @@
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220" s="4" t="s">
-        <v>205</v>
+        <v>17</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C220" s="4">
         <v>1</v>
       </c>
       <c r="D220" s="4" t="s">
-        <v>206</v>
+        <v>18</v>
       </c>
       <c r="E220" s="4" t="s">
-        <v>154</v>
+        <v>119</v>
       </c>
       <c r="F220" s="4">
         <v>1</v>
@@ -6111,19 +6101,19 @@
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222" s="4" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>132</v>
+        <v>29</v>
       </c>
       <c r="C222" s="4">
         <v>1</v>
       </c>
       <c r="D222" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E222" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="E222" s="4" t="s">
-        <v>133</v>
       </c>
       <c r="F222" s="4">
         <v>1</v>
@@ -6151,19 +6141,19 @@
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A224" s="4" t="s">
-        <v>26</v>
+        <v>175</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>200</v>
+        <v>132</v>
       </c>
       <c r="C224" s="4">
         <v>1</v>
       </c>
       <c r="D224" s="4" t="s">
-        <v>27</v>
+        <v>176</v>
       </c>
       <c r="E224" s="4" t="s">
-        <v>201</v>
+        <v>133</v>
       </c>
       <c r="F224" s="4">
         <v>1</v>
@@ -6171,19 +6161,19 @@
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A225" s="4" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C225" s="4">
         <v>1</v>
       </c>
       <c r="D225" s="4" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E225" s="4" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="F225" s="4">
         <v>1</v>
@@ -6191,19 +6181,19 @@
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A226" s="4" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C226" s="4">
         <v>1</v>
       </c>
       <c r="D226" s="4" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E226" s="4" t="s">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="F226" s="4">
         <v>1</v>
@@ -6211,19 +6201,19 @@
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A227" s="4" t="s">
-        <v>80</v>
+        <v>196</v>
       </c>
       <c r="B227" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C227" s="4">
         <v>1</v>
       </c>
       <c r="D227" s="4" t="s">
-        <v>81</v>
+        <v>197</v>
       </c>
       <c r="E227" s="4" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="F227" s="4">
         <v>1</v>
@@ -6231,19 +6221,19 @@
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
-        <v>80</v>
+        <v>198</v>
       </c>
       <c r="B228" s="4" t="s">
-        <v>207</v>
+        <v>153</v>
       </c>
       <c r="C228" s="4">
         <v>1</v>
       </c>
       <c r="D228" s="4" t="s">
-        <v>81</v>
+        <v>199</v>
       </c>
       <c r="E228" s="4" t="s">
-        <v>71</v>
+        <v>154</v>
       </c>
       <c r="F228" s="4">
         <v>1</v>
@@ -6251,19 +6241,19 @@
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A229" s="4" t="s">
-        <v>80</v>
+        <v>198</v>
       </c>
       <c r="B229" s="4" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="C229" s="4">
         <v>1</v>
       </c>
       <c r="D229" s="4" t="s">
-        <v>81</v>
+        <v>199</v>
       </c>
       <c r="E229" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F229" s="4">
         <v>1</v>
@@ -6271,19 +6261,19 @@
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A230" s="4" t="s">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>78</v>
+        <v>186</v>
       </c>
       <c r="C230" s="4">
         <v>1</v>
       </c>
       <c r="D230" s="4" t="s">
-        <v>81</v>
+        <v>201</v>
       </c>
       <c r="E230" s="4" t="s">
-        <v>79</v>
+        <v>187</v>
       </c>
       <c r="F230" s="4">
         <v>1</v>
@@ -6291,19 +6281,19 @@
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A231" s="4" t="s">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>61</v>
+        <v>144</v>
       </c>
       <c r="C231" s="4">
         <v>1</v>
       </c>
       <c r="D231" s="4" t="s">
-        <v>22</v>
+        <v>201</v>
       </c>
       <c r="E231" s="4" t="s">
-        <v>62</v>
+        <v>146</v>
       </c>
       <c r="F231" s="4">
         <v>1</v>
@@ -6311,19 +6301,19 @@
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
-        <v>20</v>
+        <v>184</v>
       </c>
       <c r="B232" s="4" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="C232" s="4">
         <v>1</v>
       </c>
       <c r="D232" s="4" t="s">
-        <v>22</v>
+        <v>185</v>
       </c>
       <c r="E232" s="4" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F232" s="4">
         <v>1</v>
@@ -6331,19 +6321,19 @@
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
       <c r="B233" s="4" t="s">
-        <v>61</v>
+        <v>186</v>
       </c>
       <c r="C233" s="4">
         <v>1</v>
       </c>
       <c r="D233" s="4" t="s">
-        <v>22</v>
+        <v>146</v>
       </c>
       <c r="E233" s="4" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="F233" s="4">
         <v>1</v>
@@ -6351,19 +6341,19 @@
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A234" s="4" t="s">
-        <v>34</v>
+        <v>147</v>
       </c>
       <c r="B234" s="4" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C234" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D234" s="4" t="s">
-        <v>36</v>
+        <v>148</v>
       </c>
       <c r="E234" s="4" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F234" s="4">
         <v>1</v>
@@ -6371,19 +6361,19 @@
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" s="4" t="s">
-        <v>34</v>
+        <v>147</v>
       </c>
       <c r="B235" s="4" t="s">
-        <v>89</v>
+        <v>188</v>
       </c>
       <c r="C235" s="4">
         <v>1</v>
       </c>
       <c r="D235" s="4" t="s">
-        <v>36</v>
+        <v>148</v>
       </c>
       <c r="E235" s="4" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="F235" s="4">
         <v>1</v>
@@ -6391,19 +6381,19 @@
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A236" s="4" t="s">
-        <v>34</v>
+        <v>147</v>
       </c>
       <c r="B236" s="4" t="s">
-        <v>208</v>
+        <v>189</v>
       </c>
       <c r="C236" s="4">
         <v>1</v>
       </c>
       <c r="D236" s="4" t="s">
-        <v>36</v>
+        <v>148</v>
       </c>
       <c r="E236" s="4" t="s">
-        <v>79</v>
+        <v>190</v>
       </c>
       <c r="F236" s="4">
         <v>1</v>
@@ -6411,19 +6401,19 @@
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A237" s="4" t="s">
-        <v>100</v>
+        <v>147</v>
       </c>
       <c r="B237" s="4" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C237" s="4">
         <v>1</v>
       </c>
       <c r="D237" s="4" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E237" s="4" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="F237" s="4">
         <v>1</v>
@@ -6431,19 +6421,19 @@
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
-        <v>100</v>
+        <v>147</v>
       </c>
       <c r="B238" s="4" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C238" s="4">
         <v>1</v>
       </c>
       <c r="D238" s="4" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E238" s="4" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="F238" s="4">
         <v>1</v>
@@ -6451,19 +6441,19 @@
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A239" s="4" t="s">
-        <v>35</v>
+        <v>147</v>
       </c>
       <c r="B239" s="4" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="C239" s="4">
         <v>1</v>
       </c>
       <c r="D239" s="4" t="s">
-        <v>37</v>
+        <v>148</v>
       </c>
       <c r="E239" s="4" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="F239" s="4">
         <v>1</v>
@@ -6471,19 +6461,19 @@
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A240" s="4" t="s">
-        <v>35</v>
+        <v>147</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>100</v>
+        <v>191</v>
       </c>
       <c r="C240" s="4">
         <v>1</v>
       </c>
       <c r="D240" s="4" t="s">
-        <v>37</v>
+        <v>148</v>
       </c>
       <c r="E240" s="4" t="s">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="F240" s="4">
         <v>1</v>
@@ -6491,19 +6481,19 @@
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A241" s="4" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="B241" s="4" t="s">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="C241" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D241" s="4" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="E241" s="4" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="F241" s="4">
         <v>1</v>
@@ -6511,19 +6501,19 @@
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A242" s="4" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="B242" s="4" t="s">
-        <v>90</v>
+        <v>12</v>
       </c>
       <c r="C242" s="4">
         <v>1</v>
       </c>
       <c r="D242" s="4" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
       <c r="E242" s="4" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="F242" s="4">
         <v>1</v>
@@ -6531,19 +6521,19 @@
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A243" s="4" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="B243" s="4" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="C243" s="4">
         <v>1</v>
       </c>
       <c r="D243" s="4" t="s">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="E243" s="4" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="F243" s="4">
         <v>1</v>
@@ -6551,19 +6541,19 @@
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A244" s="4" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="B244" s="4" t="s">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C244" s="4">
         <v>1</v>
       </c>
       <c r="D244" s="4" t="s">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="E244" s="4" t="s">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="F244" s="4">
         <v>1</v>
@@ -6591,19 +6581,19 @@
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A246" s="4" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="B246" s="4" t="s">
-        <v>80</v>
+        <v>124</v>
       </c>
       <c r="C246" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D246" s="4" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="E246" s="4" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
       <c r="F246" s="4">
         <v>1</v>
@@ -6611,19 +6601,19 @@
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A247" s="4" t="s">
-        <v>157</v>
+        <v>140</v>
       </c>
       <c r="B247" s="4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C247" s="4">
         <v>1</v>
       </c>
       <c r="D247" s="4" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="E247" s="4" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F247" s="4">
         <v>1</v>
@@ -6631,19 +6621,19 @@
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="B248" s="4" t="s">
-        <v>209</v>
+        <v>73</v>
       </c>
       <c r="C248" s="4">
         <v>1</v>
       </c>
       <c r="D248" s="4" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="E248" s="4" t="s">
-        <v>210</v>
+        <v>14</v>
       </c>
       <c r="F248" s="4">
         <v>1</v>
@@ -6671,19 +6661,19 @@
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A250" s="4" t="s">
-        <v>161</v>
+        <v>194</v>
       </c>
       <c r="B250" s="4" t="s">
-        <v>211</v>
+        <v>100</v>
       </c>
       <c r="C250" s="4">
         <v>1</v>
       </c>
       <c r="D250" s="4" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="E250" s="4" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="F250" s="4">
         <v>1</v>
@@ -6691,19 +6681,19 @@
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A251" s="4" t="s">
-        <v>161</v>
+        <v>194</v>
       </c>
       <c r="B251" s="4" t="s">
-        <v>24</v>
+        <v>178</v>
       </c>
       <c r="C251" s="4">
         <v>1</v>
       </c>
       <c r="D251" s="4" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="E251" s="4" t="s">
-        <v>15</v>
+        <v>179</v>
       </c>
       <c r="F251" s="4">
         <v>1</v>
@@ -6711,19 +6701,19 @@
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A252" s="4" t="s">
-        <v>9</v>
+        <v>194</v>
       </c>
       <c r="B252" s="4" t="s">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="C252" s="4">
         <v>1</v>
       </c>
       <c r="D252" s="4" t="s">
-        <v>11</v>
+        <v>195</v>
       </c>
       <c r="E252" s="4" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="F252" s="4">
         <v>1</v>
@@ -6731,19 +6721,19 @@
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A253" s="4" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B253" s="4" t="s">
-        <v>196</v>
+        <v>35</v>
       </c>
       <c r="C253" s="4">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D253" s="4" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="E253" s="4" t="s">
-        <v>197</v>
+        <v>37</v>
       </c>
       <c r="F253" s="4">
         <v>1</v>
@@ -6951,19 +6941,19 @@
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A264" s="4" t="s">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="B264" s="4" t="s">
-        <v>214</v>
+        <v>38</v>
       </c>
       <c r="C264" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D264" s="4" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="E264" s="4" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="F264" s="4">
         <v>1</v>
@@ -6991,19 +6981,19 @@
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A266" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B266" s="4" t="s">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C266" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D266" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E266" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="E266" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="F266" s="4">
         <v>1</v>
@@ -7011,19 +7001,19 @@
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A267" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B267" s="4" t="s">
-        <v>34</v>
+        <v>100</v>
       </c>
       <c r="C267" s="4">
         <v>1</v>
       </c>
       <c r="D267" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E267" s="4" t="s">
-        <v>36</v>
+        <v>101</v>
       </c>
       <c r="F267" s="4">
         <v>1</v>
@@ -7031,19 +7021,19 @@
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B268" s="4" t="s">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="C268" s="4">
         <v>1</v>
       </c>
       <c r="D268" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E268" s="4" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="F268" s="4">
         <v>1</v>
@@ -7051,19 +7041,19 @@
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A269" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B269" s="4" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="C269" s="4">
         <v>1</v>
       </c>
       <c r="D269" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E269" s="4" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
       <c r="F269" s="4">
         <v>1</v>
@@ -7071,19 +7061,19 @@
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A270" s="4" t="s">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="B270" s="4" t="s">
-        <v>67</v>
+        <v>136</v>
       </c>
       <c r="C270" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D270" s="4" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="E270" s="4" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="F270" s="4">
         <v>1</v>
@@ -7091,19 +7081,19 @@
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A271" s="4" t="s">
-        <v>215</v>
+        <v>100</v>
       </c>
       <c r="B271" s="4" t="s">
-        <v>216</v>
+        <v>80</v>
       </c>
       <c r="C271" s="4">
         <v>1</v>
       </c>
       <c r="D271" s="4" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="E271" s="4" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="F271" s="4">
         <v>1</v>
@@ -7111,19 +7101,19 @@
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A272" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B272" s="4" t="s">
-        <v>217</v>
+        <v>39</v>
       </c>
       <c r="C272" s="4">
         <v>1</v>
       </c>
       <c r="D272" s="4" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="E272" s="4" t="s">
-        <v>218</v>
+        <v>37</v>
       </c>
       <c r="F272" s="4">
         <v>1</v>
@@ -7231,16 +7221,16 @@
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A278" s="4" t="s">
-        <v>53</v>
+        <v>100</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>220</v>
+        <v>90</v>
       </c>
       <c r="C278" s="4">
         <v>1</v>
       </c>
       <c r="D278" s="4" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="E278" s="4" t="s">
         <v>91</v>
@@ -7251,19 +7241,19 @@
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A279" s="4" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="B279" s="4" t="s">
-        <v>221</v>
+        <v>104</v>
       </c>
       <c r="C279" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D279" s="4" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="E279" s="4" t="s">
-        <v>14</v>
+        <v>106</v>
       </c>
       <c r="F279" s="4">
         <v>1</v>
@@ -7271,19 +7261,19 @@
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A280" s="4" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="B280" s="4" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="C280" s="4">
         <v>1</v>
       </c>
       <c r="D280" s="4" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="E280" s="4" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="F280" s="4">
         <v>1</v>
@@ -7291,19 +7281,19 @@
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A281" s="4" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
       <c r="B281" s="4" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="C281" s="4">
         <v>1</v>
       </c>
       <c r="D281" s="4" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="E281" s="4" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="F281" s="4">
         <v>1</v>
@@ -7311,19 +7301,19 @@
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A282" s="4" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B282" s="4" t="s">
-        <v>222</v>
+        <v>40</v>
       </c>
       <c r="C282" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D282" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E282" s="4" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="F282" s="4">
         <v>1</v>
@@ -7411,19 +7401,19 @@
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A287" s="4" t="s">
-        <v>223</v>
+        <v>19</v>
       </c>
       <c r="B287" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C287" s="4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D287" s="4" t="s">
-        <v>224</v>
+        <v>21</v>
       </c>
       <c r="E287" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F287" s="4">
         <v>1</v>
@@ -7431,19 +7421,19 @@
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A288" s="4" t="s">
-        <v>132</v>
+        <v>19</v>
       </c>
       <c r="B288" s="4" t="s">
-        <v>155</v>
+        <v>33</v>
       </c>
       <c r="C288" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D288" s="4" t="s">
-        <v>133</v>
+        <v>21</v>
       </c>
       <c r="E288" s="4" t="s">
-        <v>119</v>
+        <v>22</v>
       </c>
       <c r="F288" s="4">
         <v>1</v>
@@ -7451,19 +7441,19 @@
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A289" s="4" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="B289" s="4" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="C289" s="4">
         <v>1</v>
       </c>
       <c r="D289" s="4" t="s">
-        <v>133</v>
+        <v>21</v>
       </c>
       <c r="E289" s="4" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="F289" s="4">
         <v>1</v>
@@ -7471,19 +7461,19 @@
     </row>
     <row r="290" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A290" s="4" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="B290" s="4" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="C290" s="4">
         <v>1</v>
       </c>
       <c r="D290" s="4" t="s">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="E290" s="4" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="F290" s="4">
         <v>1</v>
@@ -7491,19 +7481,19 @@
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A291" s="4" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="B291" s="4" t="s">
-        <v>181</v>
+        <v>209</v>
       </c>
       <c r="C291" s="4">
         <v>1</v>
       </c>
       <c r="D291" s="4" t="s">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="E291" s="4" t="s">
-        <v>182</v>
+        <v>210</v>
       </c>
       <c r="F291" s="4">
         <v>1</v>
@@ -7591,19 +7581,19 @@
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A296" s="4" t="s">
-        <v>213</v>
+        <v>161</v>
       </c>
       <c r="B296" s="4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C296" s="4">
         <v>1</v>
       </c>
       <c r="D296" s="4" t="s">
-        <v>71</v>
+        <v>162</v>
       </c>
       <c r="E296" s="4" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="F296" s="4">
         <v>1</v>
@@ -7611,19 +7601,19 @@
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A297" s="4" t="s">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="B297" s="4" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="C297" s="4">
         <v>1</v>
       </c>
       <c r="D297" s="4" t="s">
-        <v>71</v>
+        <v>162</v>
       </c>
       <c r="E297" s="4" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="F297" s="4">
         <v>1</v>
@@ -7671,19 +7661,19 @@
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A300" s="4" t="s">
-        <v>215</v>
+        <v>9</v>
       </c>
       <c r="B300" s="4" t="s">
-        <v>225</v>
+        <v>90</v>
       </c>
       <c r="C300" s="4">
         <v>1</v>
       </c>
       <c r="D300" s="4" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E300" s="4" t="s">
-        <v>182</v>
+        <v>91</v>
       </c>
       <c r="F300" s="4">
         <v>1</v>
@@ -7811,19 +7801,19 @@
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A307" s="4" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="B307" s="4" t="s">
-        <v>104</v>
+        <v>196</v>
       </c>
       <c r="C307" s="4">
         <v>1</v>
       </c>
       <c r="D307" s="4" t="s">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E307" s="4" t="s">
-        <v>106</v>
+        <v>197</v>
       </c>
       <c r="F307" s="4">
         <v>1</v>
@@ -7831,10 +7821,10 @@
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A308" s="4" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="B308" s="4" t="s">
-        <v>103</v>
+        <v>214</v>
       </c>
       <c r="C308" s="4">
         <v>1</v>
@@ -7843,7 +7833,7 @@
         <v>71</v>
       </c>
       <c r="E308" s="4" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="F308" s="4">
         <v>1</v>
@@ -7871,10 +7861,10 @@
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A310" s="4" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="B310" s="4" t="s">
-        <v>104</v>
+        <v>216</v>
       </c>
       <c r="C310" s="4">
         <v>1</v>
@@ -7891,10 +7881,10 @@
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A311" s="4" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="B311" s="4" t="s">
-        <v>127</v>
+        <v>225</v>
       </c>
       <c r="C311" s="4">
         <v>1</v>
@@ -7903,7 +7893,7 @@
         <v>71</v>
       </c>
       <c r="E311" s="4" t="s">
-        <v>14</v>
+        <v>182</v>
       </c>
       <c r="F311" s="4">
         <v>1</v>
@@ -7911,19 +7901,19 @@
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A312" s="4" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="B312" s="4" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="C312" s="4">
         <v>1</v>
       </c>
       <c r="D312" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E312" s="4" t="s">
-        <v>62</v>
+        <v>218</v>
       </c>
       <c r="F312" s="4">
         <v>1</v>
@@ -7931,19 +7921,19 @@
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A313" s="4" t="s">
-        <v>228</v>
+        <v>96</v>
       </c>
       <c r="B313" s="4" t="s">
-        <v>170</v>
+        <v>104</v>
       </c>
       <c r="C313" s="4">
         <v>1</v>
       </c>
       <c r="D313" s="4" t="s">
-        <v>172</v>
+        <v>71</v>
       </c>
       <c r="E313" s="4" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="F313" s="4">
         <v>1</v>
@@ -7951,19 +7941,19 @@
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A314" s="4" t="s">
-        <v>228</v>
+        <v>69</v>
       </c>
       <c r="B314" s="4" t="s">
-        <v>140</v>
+        <v>103</v>
       </c>
       <c r="C314" s="4">
         <v>1</v>
       </c>
       <c r="D314" s="4" t="s">
-        <v>172</v>
+        <v>71</v>
       </c>
       <c r="E314" s="4" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="F314" s="4">
         <v>1</v>
@@ -7971,19 +7961,19 @@
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A315" s="4" t="s">
-        <v>171</v>
+        <v>69</v>
       </c>
       <c r="B315" s="4" t="s">
-        <v>229</v>
+        <v>104</v>
       </c>
       <c r="C315" s="4">
         <v>1</v>
       </c>
       <c r="D315" s="4" t="s">
-        <v>172</v>
+        <v>71</v>
       </c>
       <c r="E315" s="4" t="s">
-        <v>204</v>
+        <v>106</v>
       </c>
       <c r="F315" s="4">
         <v>1</v>
@@ -7991,19 +7981,19 @@
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A316" s="4" t="s">
-        <v>126</v>
+        <v>69</v>
       </c>
       <c r="B316" s="4" t="s">
-        <v>230</v>
+        <v>127</v>
       </c>
       <c r="C316" s="4">
         <v>1</v>
       </c>
       <c r="D316" s="4" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E316" s="4" t="s">
-        <v>218</v>
+        <v>14</v>
       </c>
       <c r="F316" s="4">
         <v>1</v>
@@ -8031,19 +8021,19 @@
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A318" s="4" t="s">
-        <v>127</v>
+        <v>213</v>
       </c>
       <c r="B318" s="4" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="C318" s="4">
         <v>1</v>
       </c>
       <c r="D318" s="4" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E318" s="4" t="s">
-        <v>195</v>
+        <v>106</v>
       </c>
       <c r="F318" s="4">
         <v>1</v>
@@ -8071,19 +8061,19 @@
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A320" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B320" s="4" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C320" s="4">
         <v>1</v>
       </c>
       <c r="D320" s="4" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="E320" s="4" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="F320" s="4">
         <v>1</v>
@@ -8091,19 +8081,19 @@
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A321" s="4" t="s">
-        <v>128</v>
+        <v>167</v>
       </c>
       <c r="B321" s="4" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="C321" s="4">
         <v>1</v>
       </c>
       <c r="D321" s="4" t="s">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="E321" s="4" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="F321" s="4">
         <v>1</v>
@@ -8371,19 +8361,19 @@
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A335" s="4" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B335" s="4" t="s">
-        <v>147</v>
+        <v>90</v>
       </c>
       <c r="C335" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D335" s="4" t="s">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="E335" s="4" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
       <c r="F335" s="4">
         <v>1</v>
@@ -8411,19 +8401,19 @@
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A337" s="4" t="s">
-        <v>211</v>
+        <v>89</v>
       </c>
       <c r="B337" s="4" t="s">
-        <v>191</v>
+        <v>60</v>
       </c>
       <c r="C337" s="4">
         <v>1</v>
       </c>
       <c r="D337" s="4" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="E337" s="4" t="s">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="F337" s="4">
         <v>1</v>
@@ -8431,19 +8421,19 @@
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A338" s="4" t="s">
-        <v>211</v>
+        <v>89</v>
       </c>
       <c r="B338" s="4" t="s">
-        <v>160</v>
+        <v>231</v>
       </c>
       <c r="C338" s="4">
         <v>1</v>
       </c>
       <c r="D338" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E338" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E338" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="F338" s="4">
         <v>1</v>
@@ -8471,19 +8461,19 @@
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A340" s="4" t="s">
-        <v>167</v>
+        <v>44</v>
       </c>
       <c r="B340" s="4" t="s">
-        <v>193</v>
+        <v>232</v>
       </c>
       <c r="C340" s="4">
         <v>1</v>
       </c>
       <c r="D340" s="4" t="s">
-        <v>168</v>
+        <v>46</v>
       </c>
       <c r="E340" s="4" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="F340" s="4">
         <v>1</v>
@@ -8491,10 +8481,10 @@
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A341" s="4" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="B341" s="4" t="s">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="C341" s="4">
         <v>1</v>
@@ -8503,7 +8493,7 @@
         <v>46</v>
       </c>
       <c r="E341" s="4" t="s">
-        <v>62</v>
+        <v>139</v>
       </c>
       <c r="F341" s="4">
         <v>1</v>
@@ -8551,10 +8541,10 @@
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A344" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B344" s="4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C344" s="4">
         <v>1</v>
@@ -8563,7 +8553,7 @@
         <v>46</v>
       </c>
       <c r="E344" s="4" t="s">
-        <v>15</v>
+        <v>234</v>
       </c>
       <c r="F344" s="4">
         <v>1</v>
@@ -8571,19 +8561,19 @@
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A345" s="4" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="B345" s="4" t="s">
-        <v>232</v>
+        <v>16</v>
       </c>
       <c r="C345" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D345" s="4" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E345" s="4" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="F345" s="4">
         <v>1</v>
@@ -8591,19 +8581,19 @@
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A346" s="4" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="B346" s="4" t="s">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="C346" s="4">
         <v>1</v>
       </c>
       <c r="D346" s="4" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E346" s="4" t="s">
-        <v>139</v>
+        <v>81</v>
       </c>
       <c r="F346" s="4">
         <v>1</v>
@@ -8631,19 +8621,19 @@
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A348" s="4" t="s">
-        <v>88</v>
+        <v>128</v>
       </c>
       <c r="B348" s="4" t="s">
-        <v>233</v>
+        <v>173</v>
       </c>
       <c r="C348" s="4">
         <v>1</v>
       </c>
       <c r="D348" s="4" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E348" s="4" t="s">
-        <v>234</v>
+        <v>111</v>
       </c>
       <c r="F348" s="4">
         <v>1</v>
@@ -8731,19 +8721,19 @@
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A353" s="4" t="s">
-        <v>13</v>
+        <v>128</v>
       </c>
       <c r="B353" s="4" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="C353" s="4">
         <v>1</v>
       </c>
       <c r="D353" s="4" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E353" s="4" t="s">
-        <v>218</v>
+        <v>14</v>
       </c>
       <c r="F353" s="4">
         <v>1</v>
@@ -8791,16 +8781,16 @@
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A356" s="4" t="s">
-        <v>13</v>
+        <v>236</v>
       </c>
       <c r="B356" s="4" t="s">
-        <v>221</v>
+        <v>73</v>
       </c>
       <c r="C356" s="4">
         <v>1</v>
       </c>
       <c r="D356" s="4" t="s">
-        <v>15</v>
+        <v>237</v>
       </c>
       <c r="E356" s="4" t="s">
         <v>14</v>
@@ -8811,19 +8801,19 @@
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A357" s="4" t="s">
-        <v>221</v>
+        <v>104</v>
       </c>
       <c r="B357" s="4" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
       <c r="C357" s="4">
         <v>1</v>
       </c>
       <c r="D357" s="4" t="s">
-        <v>14</v>
+        <v>106</v>
       </c>
       <c r="E357" s="4" t="s">
-        <v>15</v>
+        <v>148</v>
       </c>
       <c r="F357" s="4">
         <v>1</v>
@@ -8851,19 +8841,19 @@
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A359" s="4" t="s">
-        <v>124</v>
+        <v>211</v>
       </c>
       <c r="B359" s="4" t="s">
-        <v>53</v>
+        <v>191</v>
       </c>
       <c r="C359" s="4">
         <v>1</v>
       </c>
       <c r="D359" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E359" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F359" s="4">
         <v>1</v>
@@ -8871,19 +8861,19 @@
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A360" s="4" t="s">
-        <v>85</v>
+        <v>211</v>
       </c>
       <c r="B360" s="4" t="s">
-        <v>211</v>
+        <v>160</v>
       </c>
       <c r="C360" s="4">
         <v>1</v>
       </c>
       <c r="D360" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E360" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F360" s="4">
         <v>1</v>
@@ -8911,16 +8901,16 @@
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A362" s="4" t="s">
-        <v>128</v>
+        <v>24</v>
       </c>
       <c r="B362" s="4" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C362" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D362" s="4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E362" s="4" t="s">
         <v>14</v>
@@ -8991,16 +8981,16 @@
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A366" s="4" t="s">
-        <v>236</v>
+        <v>24</v>
       </c>
       <c r="B366" s="4" t="s">
-        <v>73</v>
+        <v>191</v>
       </c>
       <c r="C366" s="4">
         <v>1</v>
       </c>
       <c r="D366" s="4" t="s">
-        <v>237</v>
+        <v>15</v>
       </c>
       <c r="E366" s="4" t="s">
         <v>14</v>
@@ -9011,19 +9001,19 @@
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A367" s="4" t="s">
-        <v>183</v>
+        <v>24</v>
       </c>
       <c r="B367" s="4" t="s">
-        <v>13</v>
+        <v>159</v>
       </c>
       <c r="C367" s="4">
         <v>1</v>
       </c>
       <c r="D367" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E367" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F367" s="4">
         <v>1</v>
@@ -9071,19 +9061,19 @@
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A370" s="4" t="s">
-        <v>125</v>
+        <v>24</v>
       </c>
       <c r="B370" s="4" t="s">
-        <v>24</v>
+        <v>73</v>
       </c>
       <c r="C370" s="4">
         <v>1</v>
       </c>
       <c r="D370" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E370" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F370" s="4">
         <v>1</v>
@@ -9131,19 +9121,19 @@
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A373" s="4" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="B373" s="4" t="s">
-        <v>13</v>
+        <v>230</v>
       </c>
       <c r="C373" s="4">
         <v>1</v>
       </c>
       <c r="D373" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E373" s="4" t="s">
-        <v>15</v>
+        <v>218</v>
       </c>
       <c r="F373" s="4">
         <v>1</v>
@@ -9171,19 +9161,19 @@
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A375" s="4" t="s">
-        <v>222</v>
+        <v>13</v>
       </c>
       <c r="B375" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C375" s="4">
         <v>1</v>
       </c>
       <c r="D375" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E375" s="4" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="F375" s="4">
         <v>1</v>
@@ -9251,19 +9241,19 @@
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A379" s="4" t="s">
-        <v>24</v>
+        <v>221</v>
       </c>
       <c r="B379" s="4" t="s">
-        <v>191</v>
+        <v>13</v>
       </c>
       <c r="C379" s="4">
         <v>1</v>
       </c>
       <c r="D379" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E379" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E379" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="F379" s="4">
         <v>1</v>
@@ -9271,19 +9261,19 @@
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A380" s="4" t="s">
-        <v>24</v>
+        <v>124</v>
       </c>
       <c r="B380" s="4" t="s">
-        <v>159</v>
+        <v>53</v>
       </c>
       <c r="C380" s="4">
         <v>1</v>
       </c>
       <c r="D380" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E380" s="4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F380" s="4">
         <v>1</v>
@@ -9291,19 +9281,19 @@
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A381" s="4" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="B381" s="4" t="s">
-        <v>73</v>
+        <v>211</v>
       </c>
       <c r="C381" s="4">
         <v>1</v>
       </c>
       <c r="D381" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E381" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E381" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="F381" s="4">
         <v>1</v>
@@ -9351,19 +9341,19 @@
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A384" s="4" t="s">
-        <v>238</v>
+        <v>85</v>
       </c>
       <c r="B384" s="4" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="C384" s="4">
         <v>1</v>
       </c>
       <c r="D384" s="4" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E384" s="4" t="s">
-        <v>91</v>
+        <v>15</v>
       </c>
       <c r="F384" s="4">
         <v>1</v>
@@ -9371,10 +9361,10 @@
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A385" s="4" t="s">
-        <v>73</v>
+        <v>183</v>
       </c>
       <c r="B385" s="4" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C385" s="4">
         <v>1</v>
@@ -9391,10 +9381,10 @@
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A386" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B386" s="4" t="s">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="C386" s="4">
         <v>1</v>
@@ -9403,7 +9393,7 @@
         <v>14</v>
       </c>
       <c r="E386" s="4" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="F386" s="4">
         <v>1</v>
@@ -9431,10 +9421,10 @@
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A388" s="4" t="s">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="B388" s="4" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C388" s="4">
         <v>1</v>
@@ -9443,7 +9433,7 @@
         <v>14</v>
       </c>
       <c r="E388" s="4" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="F388" s="4">
         <v>1</v>
@@ -9451,19 +9441,19 @@
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A389" s="4" t="s">
-        <v>61</v>
+        <v>222</v>
       </c>
       <c r="B389" s="4" t="s">
-        <v>20</v>
+        <v>220</v>
       </c>
       <c r="C389" s="4">
         <v>1</v>
       </c>
       <c r="D389" s="4" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E389" s="4" t="s">
-        <v>22</v>
+        <v>91</v>
       </c>
       <c r="F389" s="4">
         <v>1</v>
@@ -9511,19 +9501,19 @@
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A392" s="4" t="s">
-        <v>122</v>
+        <v>160</v>
       </c>
       <c r="B392" s="4" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="C392" s="4">
         <v>1</v>
       </c>
       <c r="D392" s="4" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E392" s="4" t="s">
-        <v>71</v>
+        <v>162</v>
       </c>
       <c r="F392" s="4">
         <v>1</v>
@@ -9551,19 +9541,19 @@
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A394" s="4" t="s">
-        <v>242</v>
+        <v>160</v>
       </c>
       <c r="B394" s="4" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="C394" s="4">
         <v>1</v>
       </c>
       <c r="D394" s="4" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E394" s="4" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="F394" s="4">
         <v>1</v>
@@ -9591,10 +9581,10 @@
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A396" s="4" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B396" s="4" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C396" s="4">
         <v>1</v>
@@ -9651,19 +9641,19 @@
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A399" s="4" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="B399" s="4" t="s">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="C399" s="4">
         <v>1</v>
       </c>
       <c r="D399" s="4" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="E399" s="4" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="F399" s="4">
         <v>1</v>
@@ -9671,19 +9661,19 @@
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A400" s="4" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="B400" s="4" t="s">
-        <v>193</v>
+        <v>13</v>
       </c>
       <c r="C400" s="4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D400" s="4" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E400" s="4" t="s">
-        <v>81</v>
+        <v>15</v>
       </c>
       <c r="F400" s="4">
         <v>1</v>
@@ -9711,19 +9701,19 @@
     </row>
     <row r="402" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A402" s="4" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B402" s="4" t="s">
-        <v>205</v>
+        <v>38</v>
       </c>
       <c r="C402" s="4">
         <v>1</v>
       </c>
       <c r="D402" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E402" s="4" t="s">
-        <v>206</v>
+        <v>37</v>
       </c>
       <c r="F402" s="4">
         <v>1</v>
@@ -9871,19 +9861,19 @@
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A410" s="4" t="s">
-        <v>208</v>
+        <v>180</v>
       </c>
       <c r="B410" s="4" t="s">
-        <v>245</v>
+        <v>151</v>
       </c>
       <c r="C410" s="4">
         <v>1</v>
       </c>
       <c r="D410" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E410" s="4" t="s">
         <v>79</v>
-      </c>
-      <c r="E410" s="4" t="s">
-        <v>246</v>
       </c>
       <c r="F410" s="4">
         <v>1</v>
@@ -9891,19 +9881,19 @@
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A411" s="4" t="s">
-        <v>208</v>
+        <v>72</v>
       </c>
       <c r="B411" s="4" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="C411" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D411" s="4" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E411" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F411" s="4">
         <v>1</v>
@@ -9951,19 +9941,19 @@
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A414" s="4" t="s">
-        <v>153</v>
+        <v>72</v>
       </c>
       <c r="B414" s="4" t="s">
-        <v>25</v>
+        <v>181</v>
       </c>
       <c r="C414" s="4">
         <v>1</v>
       </c>
       <c r="D414" s="4" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="E414" s="4" t="s">
-        <v>27</v>
+        <v>182</v>
       </c>
       <c r="F414" s="4">
         <v>1</v>
@@ -9971,19 +9961,19 @@
     </row>
     <row r="415" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A415" s="4" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="B415" s="4" t="s">
-        <v>155</v>
+        <v>53</v>
       </c>
       <c r="C415" s="4">
         <v>1</v>
       </c>
       <c r="D415" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E415" s="4" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="F415" s="4">
         <v>1</v>
@@ -9991,19 +9981,19 @@
     </row>
     <row r="416" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A416" s="4" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="B416" s="4" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C416" s="4">
         <v>1</v>
       </c>
       <c r="D416" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E416" s="4" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="F416" s="4">
         <v>1</v>
@@ -10011,19 +10001,19 @@
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A417" s="4" t="s">
-        <v>25</v>
+        <v>126</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>55</v>
+        <v>230</v>
       </c>
       <c r="C417" s="4">
         <v>1</v>
       </c>
       <c r="D417" s="4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E417" s="4" t="s">
-        <v>57</v>
+        <v>218</v>
       </c>
       <c r="F417" s="4">
         <v>1</v>
@@ -10071,19 +10061,19 @@
     </row>
     <row r="420" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A420" s="4" t="s">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="B420" s="4" t="s">
-        <v>130</v>
+        <v>194</v>
       </c>
       <c r="C420" s="4">
         <v>1</v>
       </c>
       <c r="D420" s="4" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E420" s="4" t="s">
-        <v>71</v>
+        <v>195</v>
       </c>
       <c r="F420" s="4">
         <v>1</v>
@@ -10091,10 +10081,10 @@
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A421" s="4" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="B421" s="4" t="s">
-        <v>23</v>
+        <v>129</v>
       </c>
       <c r="C421" s="4">
         <v>1</v>
@@ -10103,7 +10093,7 @@
         <v>79</v>
       </c>
       <c r="E421" s="4" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="F421" s="4">
         <v>1</v>
@@ -10131,19 +10121,19 @@
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A423" s="4" t="s">
-        <v>61</v>
+        <v>242</v>
       </c>
       <c r="B423" s="4" t="s">
-        <v>192</v>
+        <v>40</v>
       </c>
       <c r="C423" s="4">
         <v>1</v>
       </c>
       <c r="D423" s="4" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="E423" s="4" t="s">
-        <v>190</v>
+        <v>42</v>
       </c>
       <c r="F423" s="4">
         <v>1</v>
@@ -10151,19 +10141,19 @@
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A424" s="4" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B424" s="4" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C424" s="4">
         <v>1</v>
       </c>
       <c r="D424" s="4" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="E424" s="4" t="s">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="F424" s="4">
         <v>1</v>
@@ -10171,16 +10161,16 @@
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A425" s="4" t="s">
-        <v>247</v>
+        <v>150</v>
       </c>
       <c r="B425" s="4" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="C425" s="4">
         <v>1</v>
       </c>
       <c r="D425" s="4" t="s">
-        <v>248</v>
+        <v>79</v>
       </c>
       <c r="E425" s="4" t="s">
         <v>71</v>
@@ -10191,19 +10181,19 @@
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A426" s="4" t="s">
-        <v>214</v>
+        <v>150</v>
       </c>
       <c r="B426" s="4" t="s">
-        <v>113</v>
+        <v>23</v>
       </c>
       <c r="C426" s="4">
         <v>1</v>
       </c>
       <c r="D426" s="4" t="s">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E426" s="4" t="s">
-        <v>115</v>
+        <v>15</v>
       </c>
       <c r="F426" s="4">
         <v>1</v>
@@ -10211,19 +10201,19 @@
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A427" s="4" t="s">
-        <v>249</v>
+        <v>208</v>
       </c>
       <c r="B427" s="4" t="s">
-        <v>73</v>
+        <v>245</v>
       </c>
       <c r="C427" s="4">
         <v>1</v>
       </c>
       <c r="D427" s="4" t="s">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E427" s="4" t="s">
-        <v>14</v>
+        <v>246</v>
       </c>
       <c r="F427" s="4">
         <v>1</v>
@@ -10251,19 +10241,19 @@
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A429" s="4" t="s">
-        <v>152</v>
+        <v>208</v>
       </c>
       <c r="B429" s="4" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="C429" s="4">
         <v>1</v>
       </c>
       <c r="D429" s="4" t="s">
-        <v>154</v>
+        <v>79</v>
       </c>
       <c r="E429" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F429" s="4">
         <v>1</v>
@@ -10296,13 +10286,16 @@
         <filter val="1"/>
       </filters>
     </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:F429">
+      <sortCondition ref="A1:A430"/>
+    </sortState>
   </autoFilter>
   <conditionalFormatting sqref="F1:F1048576">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update .gitignore to exclude unnecessary files and directories
</commit_message>
<xml_diff>
--- a/CSVs/misclassification_distribution_with_family_flag.xlsx
+++ b/CSVs/misclassification_distribution_with_family_flag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meghp\Desktop\Ahmedabad University\Term 1\CSE618 Artificial Intelligence Laboratory\Bird Species Detection\CSVs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CB7B45-198A-4D13-8544-D516EC296CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D46F3A-710B-4B0A-BEA3-F002D7BEF9D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BE3F7B11-DE27-46EE-97E8-441B81A35EB4}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2581" uniqueCount="257">
   <si>
     <t>True Label</t>
   </si>
@@ -791,6 +791,9 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -1348,17 +1351,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="33">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1376,206 +1369,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1646,36 +1439,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2091,7 +1854,7 @@
         <v>254</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
@@ -11903,22 +11666,25 @@
       <sortCondition ref="A1:A430"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="G2">
-    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",G2)))</formula>
+  <conditionalFormatting sqref="F1:F1048576">
+    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Yes">
+      <formula>NOT(ISERROR(SEARCH("Yes",F1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="No">
+      <formula>NOT(ISERROR(SEARCH("No",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="Pending">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",G1)))</formula>
     </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",G1)))</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="No">
-      <formula>NOT(ISERROR(SEARCH("No",F1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Yes">
-      <formula>NOT(ISERROR(SEARCH("Yes",F1)))</formula>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>